<commit_message>
Kullanıcı merkezli asistan ve daha genel temizleme
- Aynı isimli farklı kişiler için 'birleştireyim mi?' sorusu, birleşince çelişen alanlar için 'hangisi doğru?'
- Soruları tek tek soran asistan balonu, atla / geri al, hücre balonu, tekrarları tek satıra indirme
- Yeni sütun türleri: unvan, fakülte, öğrenim düzeyi, cinsiyet, tarih, sayı; içerikten tür tahmini
- Ayrı Ad/Soyad sütunları, başlık satırı tespiti, Windows-1254 ve ';' ayraçlı CSV
- E-posta alan adı düzeltmesi, bilinmeyen sütunlarda tek yazıma indirme
- Yeni test senaryoları ve soruları cevaplayan sanal kullanıcı ile ölçüm

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7E9JFg7jqX1ZLRzaJSKG7
</commit_message>
<xml_diff>
--- a/tests/data/Sentetik_Agir_Kirli.xlsx
+++ b/tests/data/Sentetik_Agir_Kirli.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:J74"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +421,15 @@
       <c r="G1" t="str">
         <v>Sehir</v>
       </c>
+      <c r="H1" t="str">
+        <v>Unvan</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Cinsiyet</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Kulup</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -433,7 +442,7 @@
         <v>REBHERLİK VE PSİKOLOJİK DANİSMANLİK</v>
       </c>
       <c r="D2" t="str">
-        <v xml:space="preserve">  ADEM.SEVINC.15@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ADEM.SEVINC.15@outlook.com </v>
       </c>
       <c r="E2" t="str">
         <v>0531 807 88 47</v>
@@ -443,6 +452,15 @@
       </c>
       <c r="G2" t="str">
         <v>Zonguldak</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Arş Gör</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J2" t="str">
+        <v>DAĞCILIK KULÜBÜ</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +474,7 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v xml:space="preserve">  ERTUGRUL.GOKTAS.31@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ERTUGRUL.GOKTAS.31@hotmail.com </v>
       </c>
       <c r="E3" t="str">
         <v>0549 536 33 93</v>
@@ -466,6 +484,15 @@
       </c>
       <c r="G3" t="str">
         <v>Karabük</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Dağcılık Kulübü</v>
       </c>
     </row>
     <row r="4">
@@ -490,6 +517,15 @@
       <c r="G4" t="str">
         <v>Kastamonu</v>
       </c>
+      <c r="H4" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>K</v>
+      </c>
+      <c r="J4" t="str">
+        <v>TİYATRO KULÜBÜ</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -513,6 +549,15 @@
       <c r="G5" t="str">
         <v>Kırıkkale</v>
       </c>
+      <c r="H5" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Satranç Kulübü</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -525,7 +570,7 @@
         <v>FİZİK</v>
       </c>
       <c r="D6" t="str">
-        <v xml:space="preserve">  EYMEN.BILGIN.32@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  EYMEN.BILGIN.32@outlook.com </v>
       </c>
       <c r="E6" t="str">
         <v>5833375737</v>
@@ -535,6 +580,15 @@
       </c>
       <c r="G6" t="str">
         <v>Amasya</v>
+      </c>
+      <c r="H6" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I6" t="str">
+        <v>kadın</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Dagcilik Kulubu</v>
       </c>
     </row>
     <row r="7">
@@ -559,6 +613,15 @@
       <c r="G7" t="str">
         <v>Mugla</v>
       </c>
+      <c r="H7" t="str">
+        <v>Öğrenci</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Dağcılık Kulübü</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -571,7 +634,7 @@
         <v>Amerikan Kültürü ve Edebiyatı</v>
       </c>
       <c r="D8" t="str">
-        <v>tarik.cakmak.18@example.invalid</v>
+        <v>tarik.cakmak.18@outlok.com</v>
       </c>
       <c r="E8" t="str">
         <v>0548 610 53 14</v>
@@ -581,6 +644,15 @@
       </c>
       <c r="G8" t="str">
         <v>Ordu</v>
+      </c>
+      <c r="H8" t="str">
+        <v>ÖĞR. GÖR.</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J8" t="str">
+        <v>MÜZİK KULÜBÜ</v>
       </c>
     </row>
     <row r="9">
@@ -594,7 +666,7 @@
         <v>Siyaset Bilimi ve Uluslararası İlişkiler</v>
       </c>
       <c r="D9" t="str">
-        <v>burhan.alkan.9@example.invalid</v>
+        <v>burhan.alkan.9@outlok.com</v>
       </c>
       <c r="E9" t="str">
         <v>0545 837 22 03</v>
@@ -604,6 +676,15 @@
       </c>
       <c r="G9" t="str">
         <v>Diyarbakır</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Ogrenci</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J9" t="str">
+        <v>robotik kulübü</v>
       </c>
     </row>
     <row r="10">
@@ -617,7 +698,7 @@
         <v>Felsefe</v>
       </c>
       <c r="D10" t="str">
-        <v xml:space="preserve">  HANDE.ONDER.7@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  HANDE.ONDER.7@gmail.com </v>
       </c>
       <c r="E10" t="str">
         <v>0555 680 92 36</v>
@@ -627,6 +708,15 @@
       </c>
       <c r="G10" t="str">
         <v>Yozgat</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Müzik Kulübü</v>
       </c>
     </row>
     <row r="11">
@@ -640,7 +730,7 @@
         <v>Muzik</v>
       </c>
       <c r="D11" t="str">
-        <v>tuncay.ince.19@example.invalid</v>
+        <v>tuncay.ince.19@gmail.com</v>
       </c>
       <c r="E11" t="str">
         <v>+90 (587) 523-53-74</v>
@@ -650,6 +740,15 @@
       </c>
       <c r="G11" t="str">
         <v>ORDU</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Satranç Kulübü</v>
       </c>
     </row>
     <row r="12">
@@ -674,6 +773,15 @@
       <c r="G12" t="str">
         <v>KARAMAN</v>
       </c>
+      <c r="H12" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I12" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Dagcilik Kulubu</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -686,7 +794,7 @@
         <v>felsefe</v>
       </c>
       <c r="D13" t="str">
-        <v>hand.eonder.7@example.invalid</v>
+        <v>hand.eonder.7@gmail.com</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -696,6 +804,15 @@
       </c>
       <c r="G13" t="str">
         <v>Yozgat</v>
+      </c>
+      <c r="H13" t="str">
+        <v>ARŞ. GÖR.</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J13" t="str">
+        <v>müzik kulübü</v>
       </c>
     </row>
     <row r="14">
@@ -720,6 +837,15 @@
       <c r="G14" t="str">
         <v>Bingol</v>
       </c>
+      <c r="H14" t="str">
+        <v>Yrd. Doç. Dr.</v>
+      </c>
+      <c r="I14" t="str">
+        <v>ERKEK</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Müzik Kulbüü</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -732,7 +858,7 @@
         <v>Sanat Tarihi</v>
       </c>
       <c r="D15" t="str">
-        <v>sibel.ciftci.20@example.invalid</v>
+        <v>sibel.ciftci.20@outlook.com</v>
       </c>
       <c r="E15" t="str">
         <v>0547 853 68 44</v>
@@ -742,6 +868,15 @@
       </c>
       <c r="G15" t="str">
         <v>Kastamonu</v>
+      </c>
+      <c r="H15" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J15" t="str">
+        <v>tiyatro kulübü</v>
       </c>
     </row>
     <row r="16">
@@ -755,7 +890,7 @@
         <v>SAGLİK YONETİMİ</v>
       </c>
       <c r="D16" t="str">
-        <v>bayram.yildiz.24@example.invalid</v>
+        <v>bayram.yildiz.24@outlook.com</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -765,6 +900,15 @@
       </c>
       <c r="G16" t="str">
         <v>Nevsehir</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Dr. Ogr. Uyesi</v>
+      </c>
+      <c r="I16" t="str">
+        <v>erkek</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Satranc Kulubu</v>
       </c>
     </row>
     <row r="17">
@@ -778,7 +922,7 @@
         <v>ftr</v>
       </c>
       <c r="D17" t="str">
-        <v xml:space="preserve">  LEVENT.CANER.34@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  LEVENT.CANER.34@gmail.com </v>
       </c>
       <c r="E17" t="str">
         <v>0586 791 43 38</v>
@@ -788,6 +932,15 @@
       </c>
       <c r="G17" t="str">
         <v>VAN</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Satranç Kulübü</v>
       </c>
     </row>
     <row r="18">
@@ -801,7 +954,7 @@
         <v>COGRAFYA</v>
       </c>
       <c r="D18" t="str">
-        <v>goktug.oral.2@example.invalid</v>
+        <v>goktug.oral.2@outlook.com</v>
       </c>
       <c r="E18" t="str">
         <v>0578 956 15 28</v>
@@ -811,6 +964,15 @@
       </c>
       <c r="G18" t="str">
         <v>Istanbul</v>
+      </c>
+      <c r="H18" t="str">
+        <v>ÖĞRENCİ</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="19">
@@ -824,7 +986,7 @@
         <v>MBG</v>
       </c>
       <c r="D19" t="str">
-        <v xml:space="preserve">  ERTUGRUL.GOKTAS.31@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ERTUGRUL.GOKTAS.31@hotmial.com </v>
       </c>
       <c r="E19" t="str">
         <v>5495363393</v>
@@ -834,6 +996,15 @@
       </c>
       <c r="G19" t="str">
         <v>Karabuk</v>
+      </c>
+      <c r="H19" t="str">
+        <v>prof. dr.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>K</v>
+      </c>
+      <c r="J19" t="str">
+        <v>DAĞCILIK KULÜBÜ</v>
       </c>
     </row>
     <row r="20">
@@ -847,7 +1018,7 @@
         <v>Pilotaj</v>
       </c>
       <c r="D20" t="str">
-        <v>goktu.goral.1@example.invalid</v>
+        <v>goktu.goral.1@hotmail.com</v>
       </c>
       <c r="E20" t="str">
         <v>5408717935</v>
@@ -857,6 +1028,15 @@
       </c>
       <c r="G20" t="str">
         <v>OSMANİYE</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Girişimcilik Kulübü</v>
       </c>
     </row>
     <row r="21">
@@ -870,7 +1050,7 @@
         <v>Insan Kaynaklari Yonetimi</v>
       </c>
       <c r="D21" t="str">
-        <v xml:space="preserve">  CAN.SARI.5@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  CAN.SARI.5@outlok.com </v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -880,6 +1060,15 @@
       </c>
       <c r="G21" t="str">
         <v>NEVŞEHİR</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Ogr. Gor.</v>
+      </c>
+      <c r="I21" t="str">
+        <v>kadın</v>
+      </c>
+      <c r="J21" t="str">
+        <v>TiyatroK ulübü</v>
       </c>
     </row>
     <row r="22">
@@ -893,7 +1082,7 @@
         <v>Saglk Yoneitmi</v>
       </c>
       <c r="D22" t="str">
-        <v>bayram.yildiz.24@example.invalid</v>
+        <v>bayram.yildiz.24@outlook.com</v>
       </c>
       <c r="E22" t="str">
         <v>5935534670</v>
@@ -903,6 +1092,15 @@
       </c>
       <c r="G22" t="str">
         <v>NEVŞEHİR</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Dr. Ogr. Uyesi</v>
+      </c>
+      <c r="I22" t="str">
+        <v>E</v>
+      </c>
+      <c r="J22" t="str">
+        <v>satranç kulübü</v>
       </c>
     </row>
     <row r="23">
@@ -916,7 +1114,7 @@
         <v>Endustri Muhendisligi</v>
       </c>
       <c r="D23" t="str">
-        <v xml:space="preserve">  BURAK.AYHAN.22@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  BURAK.AYHAN.22@outlook.com </v>
       </c>
       <c r="E23" t="str">
         <v>0593 584 86 54</v>
@@ -926,6 +1124,15 @@
       </c>
       <c r="G23" t="str">
         <v>Malatya</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Profesör</v>
+      </c>
+      <c r="I23" t="str">
+        <v>E</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Tiytaro Kulübü</v>
       </c>
     </row>
     <row r="24">
@@ -950,6 +1157,15 @@
       <c r="G24" t="str">
         <v>Osmaniye</v>
       </c>
+      <c r="H24" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Girişimcilik Kulübü</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -962,7 +1178,7 @@
         <v>CGORAFYA</v>
       </c>
       <c r="D25" t="str">
-        <v xml:space="preserve">  GOKTUG.ORAL.2@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  GOKTUG.ORAL.2@outlok.com </v>
       </c>
       <c r="E25" t="str">
         <v>5789561528</v>
@@ -972,6 +1188,15 @@
       </c>
       <c r="G25" t="str">
         <v>İstanbul</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Ogrenci</v>
+      </c>
+      <c r="I25" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="26">
@@ -985,7 +1210,7 @@
         <v>sanat tarhii</v>
       </c>
       <c r="D26" t="str">
-        <v xml:space="preserve">  SIBEL.CIFTCI.20@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  SIBEL.CIFTCI.20@outlook.com </v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -995,6 +1220,15 @@
       </c>
       <c r="G26" t="str">
         <v>Kastamonu</v>
+      </c>
+      <c r="H26" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I26" t="str">
+        <v>kadın</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="27">
@@ -1019,6 +1253,15 @@
       <c r="G27" t="str">
         <v>Burdur</v>
       </c>
+      <c r="H27" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Girişimcilik Kulübü</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1042,6 +1285,15 @@
       <c r="G28" t="str">
         <v>Sakarya</v>
       </c>
+      <c r="H28" t="str">
+        <v>ÖĞRENCİ</v>
+      </c>
+      <c r="I28" t="str">
+        <v>K</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Muzik Kulubu</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1054,7 +1306,7 @@
         <v>Ekonometri</v>
       </c>
       <c r="D29" t="str">
-        <v>lavin.gunes.12@example.invalid</v>
+        <v>lavin.gunes.12@outlook.com</v>
       </c>
       <c r="E29" t="str">
         <v>0545 377 43 73</v>
@@ -1064,6 +1316,15 @@
       </c>
       <c r="G29" t="str">
         <v>Gaziantep</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Dr. Öğr. Üyesi</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Tiyatro Kulübü</v>
       </c>
     </row>
     <row r="30">
@@ -1077,7 +1338,7 @@
         <v>SOSYAL HİZMET</v>
       </c>
       <c r="D30" t="str">
-        <v>gulsen.ozgur.16@example.invalid</v>
+        <v>gulsen.ozgur.16@outlook.com</v>
       </c>
       <c r="E30" t="str">
         <v>5478938025</v>
@@ -1087,6 +1348,15 @@
       </c>
       <c r="G30" t="str">
         <v>Bilecik</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Tiyatro Kulübü</v>
       </c>
     </row>
     <row r="31">
@@ -1100,7 +1370,7 @@
         <v>Sosyal Hizmet</v>
       </c>
       <c r="D31" t="str">
-        <v>gulsen.ozgur.16@example.invalid</v>
+        <v>gulsen.ozgur.16@outlook.com</v>
       </c>
       <c r="E31" t="str">
         <v>0547 893 80 25</v>
@@ -1110,6 +1380,15 @@
       </c>
       <c r="G31" t="str">
         <v>Bilecik</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Tiyatro Kulübü</v>
       </c>
     </row>
     <row r="32">
@@ -1123,7 +1402,7 @@
         <v>Metalurji ve Malzeme Mühendisliği</v>
       </c>
       <c r="D32" t="str">
-        <v>deniz.bayram.35@example.invalid</v>
+        <v>deniz.bayram.35@outlook.com</v>
       </c>
       <c r="E32" t="str">
         <v>0572 744 30 95</v>
@@ -1133,6 +1412,15 @@
       </c>
       <c r="G32" t="str">
         <v>Ankara</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Ars. Gor.</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Satranc Kulubu</v>
       </c>
     </row>
     <row r="33">
@@ -1157,6 +1445,15 @@
       <c r="G33" t="str">
         <v>KÜTAHYA</v>
       </c>
+      <c r="H33" t="str">
+        <v>ÖĞR. GÖR.</v>
+      </c>
+      <c r="I33" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J33" t="str">
+        <v>MÜZİK KULÜBÜ</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1180,6 +1477,15 @@
       <c r="G34" t="str">
         <v>Edirne</v>
       </c>
+      <c r="H34" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Müzik Kulübü</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1192,7 +1498,7 @@
         <v/>
       </c>
       <c r="D35" t="str">
-        <v xml:space="preserve">  GOKTUG.ORAL.2@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  GOKTUG.ORAL.2@outlok.com </v>
       </c>
       <c r="E35" t="str">
         <v>+90 (578) 956-15-28</v>
@@ -1202,6 +1508,15 @@
       </c>
       <c r="G35" t="str">
         <v>İSTANBUL</v>
+      </c>
+      <c r="H35" t="str">
+        <v>ÖĞRENCİ</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J35" t="str">
+        <v>tiyatro kulübü</v>
       </c>
     </row>
     <row r="36">
@@ -1215,7 +1530,7 @@
         <v/>
       </c>
       <c r="D36" t="str">
-        <v xml:space="preserve">  TUNCAY.INCE.19@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  TUNCAY.INCE.19@gmail.com </v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -1225,6 +1540,15 @@
       </c>
       <c r="G36" t="str">
         <v>ORDU</v>
+      </c>
+      <c r="H36" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I36" t="str">
+        <v>K</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Satranc Kulubu</v>
       </c>
     </row>
     <row r="37">
@@ -1238,7 +1562,7 @@
         <v>JEOFİZK MUH.</v>
       </c>
       <c r="D37" t="str">
-        <v xml:space="preserve">  LEVENT.CANER.4@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  LEVENT.CANER.4@gmail.com </v>
       </c>
       <c r="E37" t="str">
         <v>5575026628</v>
@@ -1248,6 +1572,15 @@
       </c>
       <c r="G37" t="str">
         <v>KARS</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Tiyatro Kulübü</v>
       </c>
     </row>
     <row r="38">
@@ -1261,7 +1594,7 @@
         <v>FİZYOTERAPİ VE REHABİLİTASYON</v>
       </c>
       <c r="D38" t="str">
-        <v>levent.caner.34@example.invalid</v>
+        <v>levent.caner.34@gmail.con</v>
       </c>
       <c r="E38" t="str">
         <v>5867914338</v>
@@ -1271,6 +1604,15 @@
       </c>
       <c r="G38" t="str">
         <v>Van</v>
+      </c>
+      <c r="H38" t="str">
+        <v>ARŞ. GÖR.</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Satraçn Kulübü</v>
       </c>
     </row>
     <row r="39">
@@ -1295,6 +1637,15 @@
       <c r="G39" t="str">
         <v>OSMANİYE</v>
       </c>
+      <c r="H39" t="str">
+        <v>Profesör</v>
+      </c>
+      <c r="I39" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J39" t="str">
+        <v>GİRİŞİMCİLİK KULÜBÜ</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1318,6 +1669,15 @@
       <c r="G40" t="str">
         <v>Batman</v>
       </c>
+      <c r="H40" t="str">
+        <v>Yrd. Doç. Dr.</v>
+      </c>
+      <c r="I40" t="str">
+        <v>ERKEK</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Müzik Kulsbü</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1330,7 +1690,7 @@
         <v>ASTRONOMİ VE UZAY BİLİMLERİ</v>
       </c>
       <c r="D41" t="str">
-        <v xml:space="preserve">  FATIH.TUNC.25@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  FATIH.TUNC.25@outlook.com </v>
       </c>
       <c r="E41" t="str">
         <v>5688669305</v>
@@ -1340,6 +1700,15 @@
       </c>
       <c r="G41" t="str">
         <v>Çorum</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Müzik Kulübü</v>
       </c>
     </row>
     <row r="42">
@@ -1353,7 +1722,7 @@
         <v>astronomi ve uzay bilimleri</v>
       </c>
       <c r="D42" t="str">
-        <v>fati.htunc.25@example.invalid</v>
+        <v>fati.htunc.25@outlok.com</v>
       </c>
       <c r="E42" t="str">
         <v>0568 866 93 05</v>
@@ -1363,6 +1732,15 @@
       </c>
       <c r="G42" t="str">
         <v>Çorum</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Doçent</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J42" t="str">
+        <v>müzik kulübü</v>
       </c>
     </row>
     <row r="43">
@@ -1387,6 +1765,15 @@
       <c r="G43" t="str">
         <v>AYDIN</v>
       </c>
+      <c r="H43" t="str">
+        <v>Ogrenci</v>
+      </c>
+      <c r="I43" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Robotik Kulubu</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1410,6 +1797,15 @@
       <c r="G44" t="str">
         <v>ANKARA</v>
       </c>
+      <c r="H44" t="str">
+        <v>ARŞ. GÖR.</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J44" t="str">
+        <v>satranç kulübü</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -1422,7 +1818,7 @@
         <v>Fizik Müh.</v>
       </c>
       <c r="D45" t="str">
-        <v xml:space="preserve">  BUSE.OZER.26@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  BUSE.OZER.26@outlook.com </v>
       </c>
       <c r="E45" t="str">
         <v>5883154132</v>
@@ -1432,6 +1828,15 @@
       </c>
       <c r="G45" t="str">
         <v>EDİRNE</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Prof. Dr.</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Müzik Kulübü</v>
       </c>
     </row>
     <row r="46">
@@ -1445,7 +1850,7 @@
         <v>MÜZİK</v>
       </c>
       <c r="D46" t="str">
-        <v xml:space="preserve">  TUNCAY.INCE.19@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  TUNCAY.INCE.19@gmial.com </v>
       </c>
       <c r="E46" t="str">
         <v>+90 (587) 523-53-74</v>
@@ -1455,6 +1860,15 @@
       </c>
       <c r="G46" t="str">
         <v>ORDU</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Doc. Dr.</v>
+      </c>
+      <c r="I46" t="str">
+        <v>K</v>
+      </c>
+      <c r="J46" t="str">
+        <v>satranç kulübü</v>
       </c>
     </row>
     <row r="47">
@@ -1479,6 +1893,15 @@
       <c r="G47" t="str">
         <v>Bartin</v>
       </c>
+      <c r="H47" t="str">
+        <v>Prof Dr</v>
+      </c>
+      <c r="I47" t="str">
+        <v>E</v>
+      </c>
+      <c r="J47" t="str">
+        <v>tiyatro kulübü</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1491,7 +1914,7 @@
         <v>PDR</v>
       </c>
       <c r="D48" t="str">
-        <v xml:space="preserve">  ADEM.SEVINC.15@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ADEM.SEVINC.15@outlook.com </v>
       </c>
       <c r="E48" t="str">
         <v>+90 (531) 807-88-47</v>
@@ -1501,6 +1924,15 @@
       </c>
       <c r="G48" t="str">
         <v>Zonguldak</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Dağcılık Kulübü</v>
       </c>
     </row>
     <row r="49">
@@ -1514,7 +1946,7 @@
         <v>Coğrafya</v>
       </c>
       <c r="D49" t="str">
-        <v>serife.goktas.3@example.invalid</v>
+        <v>serife.goktas.3@outlook.com</v>
       </c>
       <c r="E49" t="str">
         <v>0551 912 87 40</v>
@@ -1524,6 +1956,15 @@
       </c>
       <c r="G49" t="str">
         <v>Sakarya</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Öğrenci</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Müzik Kulübü</v>
       </c>
     </row>
     <row r="50">
@@ -1537,7 +1978,7 @@
         <v>SOSYAL HİZMET</v>
       </c>
       <c r="D50" t="str">
-        <v xml:space="preserve">  GULSEN.OZGUR.16@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  GULSEN.OZGUR.16@outlok.com </v>
       </c>
       <c r="E50" t="str">
         <v>0547 893 80 25</v>
@@ -1547,6 +1988,15 @@
       </c>
       <c r="G50" t="str">
         <v>Bilecik</v>
+      </c>
+      <c r="H50" t="str">
+        <v>PROF. DR.</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="51">
@@ -1571,6 +2021,15 @@
       <c r="G51" t="str">
         <v>MALATYA</v>
       </c>
+      <c r="H51" t="str">
+        <v>Prof Dr</v>
+      </c>
+      <c r="I51" t="str">
+        <v>E</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Tiyatro Kulubu</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1583,7 +2042,7 @@
         <v>SPOR YÖNETİCİLİĞİ</v>
       </c>
       <c r="D52" t="str">
-        <v>onu.rergun.33@example.invalid</v>
+        <v>onu.rergun.33@gmail.com</v>
       </c>
       <c r="E52" t="str">
         <v>0587 596 02 05</v>
@@ -1593,6 +2052,15 @@
       </c>
       <c r="G52" t="str">
         <v>BİNGÖL</v>
+      </c>
+      <c r="H52" t="str">
+        <v>ÖĞR. GÖR.</v>
+      </c>
+      <c r="I52" t="str">
+        <v>E</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="53">
@@ -1606,7 +2074,7 @@
         <v>rekreasyon yonetimi</v>
       </c>
       <c r="D53" t="str">
-        <v xml:space="preserve">  ORHAN.DURAN.6@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ORHAN.DURAN.6@hotmail.com </v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -1616,6 +2084,15 @@
       </c>
       <c r="G53" t="str">
         <v>AKSARAY</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Dr. Ogr. Uyesi</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J53" t="str">
+        <v>MÜZİK KULÜBÜ</v>
       </c>
     </row>
     <row r="54">
@@ -1629,7 +2106,7 @@
         <v>Psikoloji</v>
       </c>
       <c r="D54" t="str">
-        <v>yunus.ozgen.28@example.invalid</v>
+        <v>yunus.ozgen.28@gmal.com</v>
       </c>
       <c r="E54" t="str">
         <v>0539 499 50 72</v>
@@ -1639,6 +2116,15 @@
       </c>
       <c r="G54" t="str">
         <v>Gaziantep</v>
+      </c>
+      <c r="H54" t="str">
+        <v>ÖĞRENCİ</v>
+      </c>
+      <c r="I54" t="str">
+        <v>ERKEK</v>
+      </c>
+      <c r="J54" t="str">
+        <v>tiyatro kulübü</v>
       </c>
     </row>
     <row r="55">
@@ -1663,6 +2149,15 @@
       <c r="G55" t="str">
         <v>KARAMAN</v>
       </c>
+      <c r="H55" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Bayan</v>
+      </c>
+      <c r="J55" t="str">
+        <v>ROBOTİK KULÜBÜ</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -1675,7 +2170,7 @@
         <v>Siyaset Bilimi ve Uluslararasi Iliskiler</v>
       </c>
       <c r="D56" t="str">
-        <v xml:space="preserve">  BURHAN.ALKAN.9@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  BURHAN.ALKAN.9@outlook.com </v>
       </c>
       <c r="E56" t="str">
         <v>+90 (545) 837-22-03</v>
@@ -1685,6 +2180,15 @@
       </c>
       <c r="G56" t="str">
         <v>Diyarbakir</v>
+      </c>
+      <c r="H56" t="str">
+        <v>ogrenci</v>
+      </c>
+      <c r="I56" t="str">
+        <v>E</v>
+      </c>
+      <c r="J56" t="str">
+        <v>ROBOTİK KULÜBÜ</v>
       </c>
     </row>
     <row r="57">
@@ -1698,7 +2202,7 @@
         <v/>
       </c>
       <c r="D57" t="str">
-        <v>levent.caner.34@example.invalid</v>
+        <v>levent.caner.34@gmail.com</v>
       </c>
       <c r="E57" t="str">
         <v>+90 (586) 791-43-38</v>
@@ -1708,6 +2212,15 @@
       </c>
       <c r="G57" t="str">
         <v>VAN</v>
+      </c>
+      <c r="H57" t="str">
+        <v>ARŞ. GÖR.</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Satranç ulübü</v>
       </c>
     </row>
     <row r="58">
@@ -1721,7 +2234,7 @@
         <v>Beslenme ve Diyetetik</v>
       </c>
       <c r="D58" t="str">
-        <v>kevser.ozkan.13@example.invalid</v>
+        <v>kevser.ozkan.13@hotmail.com</v>
       </c>
       <c r="E58" t="str">
         <v>5593362805</v>
@@ -1731,6 +2244,15 @@
       </c>
       <c r="G58" t="str">
         <v>Kırşehir</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Robotik Kulübü</v>
       </c>
     </row>
     <row r="59">
@@ -1744,7 +2266,7 @@
         <v/>
       </c>
       <c r="D59" t="str">
-        <v>hande.onder.7@example.invalid</v>
+        <v>hande.onder.7@gmail.com</v>
       </c>
       <c r="E59" t="str">
         <v>5556809236</v>
@@ -1754,6 +2276,15 @@
       </c>
       <c r="G59" t="str">
         <v>Yozgat</v>
+      </c>
+      <c r="H59" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Müzik Kulübü</v>
       </c>
     </row>
     <row r="60">
@@ -1767,7 +2298,7 @@
         <v>İnsan Kaynakları Yönetimi</v>
       </c>
       <c r="D60" t="str">
-        <v xml:space="preserve">  CAN.SARI.5@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  CAN.SARI.5@outlook.com </v>
       </c>
       <c r="E60" t="str">
         <v>5626126531</v>
@@ -1777,6 +2308,15 @@
       </c>
       <c r="G60" t="str">
         <v>NEVŞEHİR</v>
+      </c>
+      <c r="H60" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Tiyatro Kulübü</v>
       </c>
     </row>
     <row r="61">
@@ -1790,7 +2330,7 @@
         <v>Gemi İnşaatı ve Gemi Makineleri Mühendisliği</v>
       </c>
       <c r="D61" t="str">
-        <v>levent.caner.8@example.invalid</v>
+        <v>levent.caner.8@outlook.com</v>
       </c>
       <c r="E61" t="str">
         <v>0553 148 29 37</v>
@@ -1800,6 +2340,15 @@
       </c>
       <c r="G61" t="str">
         <v>Burdur</v>
+      </c>
+      <c r="H61" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Girişimcilik Kulübü</v>
       </c>
     </row>
     <row r="62">
@@ -1813,7 +2362,7 @@
         <v>otomotiv muh.</v>
       </c>
       <c r="D62" t="str">
-        <v xml:space="preserve">  SUKRU.CAN.17@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  SUKRU.CAN.17@gmail.com </v>
       </c>
       <c r="E62" t="str">
         <v>0556 428 60 44</v>
@@ -1823,6 +2372,15 @@
       </c>
       <c r="G62" t="str">
         <v>Karaman</v>
+      </c>
+      <c r="H62" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Robotik Kulübü</v>
       </c>
     </row>
     <row r="63">
@@ -1836,7 +2394,7 @@
         <v>otomotiv müh.</v>
       </c>
       <c r="D63" t="str">
-        <v>sukru.can.17@example.invalid</v>
+        <v>sukru.can.17@gmial.com</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -1846,6 +2404,15 @@
       </c>
       <c r="G63" t="str">
         <v>Karaman</v>
+      </c>
+      <c r="H63" t="str">
+        <v>Doc. Dr.</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J63" t="str">
+        <v>Robotik Kulubu</v>
       </c>
     </row>
     <row r="64">
@@ -1859,7 +2426,7 @@
         <v>GEMİ INSAATİ VE GEMİ MAKİNELERİ MUH.</v>
       </c>
       <c r="D64" t="str">
-        <v>kevser.ozkan.27@example.invalid</v>
+        <v>kevser.ozkan.27@outlok.com</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -1869,6 +2436,15 @@
       </c>
       <c r="G64" t="str">
         <v>Karaman</v>
+      </c>
+      <c r="H64" t="str">
+        <v>DOÇ. DR.</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Dağcılk Kulübü</v>
       </c>
     </row>
     <row r="65">
@@ -1882,7 +2458,7 @@
         <v>Psikoloji</v>
       </c>
       <c r="D65" t="str">
-        <v>sukru.can.14@example.invalid</v>
+        <v>sukru.can.14@gmail.com</v>
       </c>
       <c r="E65" t="str">
         <v>0571 306 25 51</v>
@@ -1892,6 +2468,15 @@
       </c>
       <c r="G65" t="str">
         <v>Kırıkkale</v>
+      </c>
+      <c r="H65" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Satranç Kulübü</v>
       </c>
     </row>
     <row r="66">
@@ -1905,7 +2490,7 @@
         <v>Fizik</v>
       </c>
       <c r="D66" t="str">
-        <v>eymen.bilgin.32@example.invalid</v>
+        <v>eymen.bilgin.32@outlook.com</v>
       </c>
       <c r="E66" t="str">
         <v>0583 337 57 37</v>
@@ -1915,6 +2500,15 @@
       </c>
       <c r="G66" t="str">
         <v>Amasya</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Doç. Dr.</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Kadın</v>
+      </c>
+      <c r="J66" t="str">
+        <v>Dağcılık Kulübü</v>
       </c>
     </row>
     <row r="67">
@@ -1928,7 +2522,7 @@
         <v>EKONOMETRİ</v>
       </c>
       <c r="D67" t="str">
-        <v xml:space="preserve">  LAVIN.GUNES.12@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  LAVIN.GUNES.12@outlok.com </v>
       </c>
       <c r="E67" t="str">
         <v>0545 377 43 73</v>
@@ -1938,6 +2532,15 @@
       </c>
       <c r="G67" t="str">
         <v>GAZİANTEP</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Yrd. Doç. Dr.</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Tiyatro Kulubu</v>
       </c>
     </row>
     <row r="68">
@@ -1951,7 +2554,7 @@
         <v>Maliye</v>
       </c>
       <c r="D68" t="str">
-        <v>yunu.sozgen.23@example.invalid</v>
+        <v>yunu.sozgen.23@hotmail.com</v>
       </c>
       <c r="E68" t="str">
         <v>+90 (577) 506-11-36</v>
@@ -1961,6 +2564,15 @@
       </c>
       <c r="G68" t="str">
         <v>Aydin</v>
+      </c>
+      <c r="H68" t="str">
+        <v>ogrenci</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Kadin</v>
+      </c>
+      <c r="J68" t="str">
+        <v>ROBOTİK KULÜBÜ</v>
       </c>
     </row>
     <row r="69">
@@ -1985,6 +2597,15 @@
       <c r="G69" t="str">
         <v>Burdur</v>
       </c>
+      <c r="H69" t="str">
+        <v>Öğr. Gör.</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Girişimcilik Kulübü</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -1997,7 +2618,7 @@
         <v>saglik yonetimi</v>
       </c>
       <c r="D70" t="str">
-        <v>bayram.yildiz.24@example.invalid</v>
+        <v>bayram.yildiz.24@outlook.com</v>
       </c>
       <c r="E70" t="str">
         <v>0593 553 46 70</v>
@@ -2007,6 +2628,15 @@
       </c>
       <c r="G70" t="str">
         <v>NEVŞEHİR</v>
+      </c>
+      <c r="H70" t="str">
+        <v>Dr. Öğr. Üyesi</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J70" t="str">
+        <v>Satranç Kulübü</v>
       </c>
     </row>
     <row r="71">
@@ -2031,6 +2661,15 @@
       <c r="G71" t="str">
         <v>GAZİANTEP</v>
       </c>
+      <c r="H71" t="str">
+        <v>Yrd. Doç. Dr.</v>
+      </c>
+      <c r="I71" t="str">
+        <v>E</v>
+      </c>
+      <c r="J71" t="str">
+        <v>tiyatro kulübü</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2043,7 +2682,7 @@
         <v>Orman Muhendisligi</v>
       </c>
       <c r="D72" t="str">
-        <v xml:space="preserve">  LEVENT.CANER.10@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  LEVENT.CANER.10@hotmail.co </v>
       </c>
       <c r="E72" t="str">
         <v>+90 (587) 596-74-32</v>
@@ -2053,6 +2692,15 @@
       </c>
       <c r="G72" t="str">
         <v>KÜTAHYA</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Öğretim Görevlisi</v>
+      </c>
+      <c r="I72" t="str">
+        <v>KADIN</v>
+      </c>
+      <c r="J72" t="str">
+        <v>Muzik Kulubu</v>
       </c>
     </row>
     <row r="73">
@@ -2066,7 +2714,7 @@
         <v>PİLOTAJ</v>
       </c>
       <c r="D73" t="str">
-        <v xml:space="preserve">  SERKAN.ERKOC.11@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  SERKAN.ERKOC.11@hotmail.com </v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -2076,6 +2724,15 @@
       </c>
       <c r="G73" t="str">
         <v>Batman</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Dr. Ogr. Uyesi</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Bay</v>
+      </c>
+      <c r="J73" t="str">
+        <v>müzik kulübü</v>
       </c>
     </row>
     <row r="74">
@@ -2089,7 +2746,7 @@
         <v/>
       </c>
       <c r="D74" t="str">
-        <v xml:space="preserve">  ADEM.SEVINC.15@EXAMPLE.INVALID </v>
+        <v xml:space="preserve">  ADEM.SEVINC.15@outlook.com </v>
       </c>
       <c r="E74" t="str">
         <v>5318078847</v>
@@ -2100,10 +2757,19 @@
       <c r="G74" t="str">
         <v>Zonguldak</v>
       </c>
+      <c r="H74" t="str">
+        <v>Arş. Gör.</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Erkek</v>
+      </c>
+      <c r="J74" t="str">
+        <v>Dağcılık Kulübü</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J74"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>